<commit_message>
Updated BOM and place files for DAQ Board
</commit_message>
<xml_diff>
--- a/PCB/DAQBoardFront/BOM.xlsx
+++ b/PCB/DAQBoardFront/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a56d338d63da0fa/Desktop/CFR-2027/PCB/DAQBoardFront/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{672BEF6D-422F-477B-B486-B83020C6D7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41A51212-5B7F-41DC-B0BA-A5BAE42F5C93}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{672BEF6D-422F-477B-B486-B83020C6D7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85C3347C-4C5D-4774-970B-FD6824BFD577}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{93B5DAD3-BF6B-4E2E-A13F-1D74895200EB}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="94">
   <si>
     <t>Designator</t>
   </si>
@@ -92,9 +92,6 @@
     <t>C_1206_3216Metric_Pad1.33x1.80mm_HandSolder</t>
   </si>
   <si>
-    <t>C3216X5R1E476M160AC</t>
-  </si>
-  <si>
     <t>D2, D3, D4</t>
   </si>
   <si>
@@ -285,6 +282,57 @@
   </si>
   <si>
     <t>C1592</t>
+  </si>
+  <si>
+    <t>C19659</t>
+  </si>
+  <si>
+    <t>C76659</t>
+  </si>
+  <si>
+    <t>C3216X5R1E476MTJ00E</t>
+  </si>
+  <si>
+    <t>C2128</t>
+  </si>
+  <si>
+    <t>C5210749</t>
+  </si>
+  <si>
+    <t>C76742</t>
+  </si>
+  <si>
+    <t>C2847484</t>
+  </si>
+  <si>
+    <t>C22846</t>
+  </si>
+  <si>
+    <t>C23352</t>
+  </si>
+  <si>
+    <t>C445827</t>
+  </si>
+  <si>
+    <t>C191552</t>
+  </si>
+  <si>
+    <t>C402975</t>
+  </si>
+  <si>
+    <t>C269673</t>
+  </si>
+  <si>
+    <t>C43473</t>
+  </si>
+  <si>
+    <t>C54968</t>
+  </si>
+  <si>
+    <t>C126014</t>
+  </si>
+  <si>
+    <t>C411212</t>
   </si>
 </sst>
 </file>
@@ -667,7 +715,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -676,12 +724,12 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -690,12 +738,12 @@
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -704,7 +752,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -728,10 +776,13 @@
       <c r="C5" t="s">
         <v>9</v>
       </c>
+      <c r="D5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>79</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
@@ -739,258 +790,303 @@
       <c r="C6" t="s">
         <v>12</v>
       </c>
+      <c r="D6" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
         <v>14</v>
       </c>
-      <c r="C7" t="s">
-        <v>15</v>
+      <c r="D7" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
         <v>17</v>
       </c>
-      <c r="C8" t="s">
-        <v>18</v>
+      <c r="D8" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
         <v>20</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
         <v>23</v>
-      </c>
-      <c r="C10" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
         <v>26</v>
       </c>
-      <c r="C11" t="s">
-        <v>27</v>
+      <c r="D11" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" t="s">
         <v>31</v>
       </c>
-      <c r="C13" t="s">
-        <v>32</v>
+      <c r="D13" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
         <v>34</v>
       </c>
-      <c r="C14" t="s">
-        <v>35</v>
+      <c r="D14" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" t="s">
         <v>41</v>
       </c>
-      <c r="B16" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="C17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" t="s">
         <v>43</v>
       </c>
-      <c r="B17" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" t="s">
         <v>46</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C19" t="s">
         <v>44</v>
       </c>
-      <c r="C18" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="D19" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" t="s">
         <v>48</v>
       </c>
-      <c r="B19" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="C20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" t="s">
         <v>50</v>
       </c>
-      <c r="B20" t="s">
-        <v>49</v>
-      </c>
-      <c r="C20" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="C21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>55</v>
+      </c>
+      <c r="B22" t="s">
         <v>53</v>
       </c>
-      <c r="B21" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="C22" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23" t="s">
         <v>56</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C23" t="s">
         <v>54</v>
       </c>
-      <c r="C22" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="D23" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" t="s">
         <v>58</v>
       </c>
-      <c r="B23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C23" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="C24" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" t="s">
         <v>60</v>
       </c>
-      <c r="B24" t="s">
-        <v>59</v>
-      </c>
-      <c r="C24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>61</v>
       </c>
-      <c r="C25" t="s">
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>22</v>
-      </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>63</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>65</v>
       </c>
-      <c r="C27" t="s">
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>22</v>
-      </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>67</v>
       </c>
-      <c r="C28" t="s">
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>70</v>
+      </c>
+      <c r="B29" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>71</v>
-      </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>69</v>
       </c>
-      <c r="C29" t="s">
-        <v>70</v>
+      <c r="D29" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>